<commit_message>
Ajustes de inicio de sesión
</commit_message>
<xml_diff>
--- a/src/test/resources/data/Usuario2.xlsx
+++ b/src/test/resources/data/Usuario2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\38513959\Downloads\SaldoLineas\SaldoLineas\src\test\resources\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pruebas\Documents\Portal-E-N\src\test\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6A31B2A-CAB2-4DF1-B601-B5A2067EA1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA7124A4-180A-42E2-B0BA-C3635D297A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,11 @@
     <sheet name="Datos" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -31,10 +36,10 @@
     <t>Numero</t>
   </si>
   <si>
-    <t>lorena.rodriguez@claro.com.co</t>
+    <t>exussmarttester@gmail.com</t>
   </si>
   <si>
-    <t>Pruebas2026*</t>
+    <t>PruebasExus2026*</t>
   </si>
 </sst>
 </file>
@@ -129,9 +134,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -169,9 +174,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -204,9 +209,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -239,9 +261,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>

</xml_diff>